<commit_message>
Mise à jour des modèles métier sections et entrées ae46a8b2b666229eed857b1d0360f4ed69d175cf
</commit_message>
<xml_diff>
--- a/htr-Corps-ModeleMetier/ig/StructureDefinition-CorpsDocument.xlsx
+++ b/htr-Corps-ModeleMetier/ig/StructureDefinition-CorpsDocument.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1623" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1530" uniqueCount="215">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-06T12:29:55+00:00</t>
+    <t>2025-10-13T08:32:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -250,7 +250,7 @@
     <t>CorpsDocument.allergiesEtHypersensibilites</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/AllergiesEtHypersensibilites
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrAllergiesEtHypersensibilites
 </t>
   </si>
   <si>
@@ -260,7 +260,7 @@
     <t>CorpsDocument.antecedentsFamiliaux</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/AntecedentsFamiliaux
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrAntecedentsFamiliaux
 </t>
   </si>
   <si>
@@ -270,7 +270,7 @@
     <t>CorpsDocument.antecedentsMedicaux</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/AntecedentsMedicaux
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrAntecedentsMedicaux
 </t>
   </si>
   <si>
@@ -280,7 +280,7 @@
     <t>CorpsDocument.codesAbarres</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/CodesAbarres
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrCodesAbarres
 </t>
   </si>
   <si>
@@ -290,7 +290,7 @@
     <t>CorpsDocument.commentaireNonCode</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/CommentaireNonCode
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrCommentaireNonCode
 </t>
   </si>
   <si>
@@ -300,7 +300,7 @@
     <t>CorpsDocument.cRBIOChapitre</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/CRBIOChapitre
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrCRBIOChapitre
 </t>
   </si>
   <si>
@@ -310,427 +310,397 @@
     <t>CorpsDocument.cRBIOSousChapitre</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/CRBIOSousChapitre
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrCRBIOSousChapitre
 </t>
   </si>
   <si>
     <t>Section Sous-chapitre du compte rendu d'examens de biologie  (section de 2nd niveau)</t>
   </si>
   <si>
-    <t>CorpsDocument.dicomActeImagerie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMActeImagerie
+    <t>CorpsDocument.acteImagerie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrActeImagerie
 </t>
   </si>
   <si>
-    <t>Section DICOM Acte d'imagerie</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomAddendum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMAddendum
+    <t>Section Acte d'imagerie</t>
+  </si>
+  <si>
+    <t>CorpsDocument.addendum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrAddendum
 </t>
   </si>
   <si>
-    <t>Section DICOM Addendum</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomConclusions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMConclusions
+    <t>Section Addendum</t>
+  </si>
+  <si>
+    <t>CorpsDocument.conclusions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrConclusionExamenImagerie
 </t>
   </si>
   <si>
-    <t>Section DICOM Conclusions</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomDemandeExamen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMDemandeExamen
+    <t>Section Conclusions</t>
+  </si>
+  <si>
+    <t>CorpsDocument.demandeExamenImagerie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDemandeExamenImagerie
 </t>
   </si>
   <si>
-    <t>Section DICOM Demande d'examen</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomExamenComparatif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMExamenComparatif
+    <t>Section Demande d'examen</t>
+  </si>
+  <si>
+    <t>CorpsDocument.comparaisonExamensImagerie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrComparaisonExamensImagerie
 </t>
   </si>
   <si>
-    <t>Section DICOM Examen comparatif</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomResultats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMResultats
+    <t>Section Examen comparatif</t>
+  </si>
+  <si>
+    <t>CorpsDocument.expositionRadiations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrExpositionRadiations
 </t>
   </si>
   <si>
-    <t>Section DICOM Résultats</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomMotifActe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMMotifActe
+    <t>Section Exposition aux radiations</t>
+  </si>
+  <si>
+    <t>CorpsDocument.informationsCliniques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrInformationsCliniques
 </t>
   </si>
   <si>
-    <t>Section DICOM Motif de l'acte</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomExpositionRadiations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMExpositionRadiations
+    <t>Section Informations cliniques</t>
+  </si>
+  <si>
+    <t>CorpsDocument.objectCatalog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrObjectCatalog
 </t>
   </si>
   <si>
-    <t>Section DICOM Exposition aux radiations</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomHistoriqueMedical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMHistoriqueMedical
+    <t>Section  Object catalog</t>
+  </si>
+  <si>
+    <t>CorpsDocument.directivesAnticipees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDirectivesAnticipees
 </t>
   </si>
   <si>
-    <t>Section DICOM Historique médical</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomInformationsCliniques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMInformationsCliniques
+    <t>Section Directives anticipées</t>
+  </si>
+  <si>
+    <t>CorpsDocument.dispensationMedicaments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDispensationMedicaments
 </t>
   </si>
   <si>
-    <t>Section DICOM Informations cliniques</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dicomObjectCatalog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DICOMObjectCatalog
+    <t>Section Dispensation médicaments</t>
+  </si>
+  <si>
+    <t>CorpsDocument.dispositifsMedicaux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDispositifsMedicaux
 </t>
   </si>
   <si>
-    <t>Section DICOM Object catalog</t>
-  </si>
-  <si>
-    <t>CorpsDocument.directivesAnticipees</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DirectivesAnticipees
+    <t>Section Dispositifs medicaux</t>
+  </si>
+  <si>
+    <t>CorpsDocument.documentPDFCopie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDocumentPDFCopie
 </t>
   </si>
   <si>
-    <t>Section Directives anticipées</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dispensationMedicaments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DispensationMedicaments
+    <t>Section Document PDF Copie</t>
+  </si>
+  <si>
+    <t>CorpsDocument.documentsAjoutes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrDocumentsAjoutes
 </t>
   </si>
   <si>
-    <t>Section Dispensation médicaments</t>
-  </si>
-  <si>
-    <t>CorpsDocument.dispositifsMedicaux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DispositifsMedicaux
+    <t>Section Documents ajoutés</t>
+  </si>
+  <si>
+    <t>CorpsDocument.educationPatient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrEducationPatient
 </t>
   </si>
   <si>
-    <t>Section Dispositifs medicaux</t>
-  </si>
-  <si>
-    <t>CorpsDocument.documentPDFCopie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DocumentPDFCopie
+    <t>Section Education du patient</t>
+  </si>
+  <si>
+    <t>CorpsDocument.effetsIndesirables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrEffetsIndesirables
 </t>
   </si>
   <si>
-    <t>Section Document PDF Copie</t>
-  </si>
-  <si>
-    <t>CorpsDocument.documentsAjoutes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/DocumentsAjoutes
+    <t>Section Effets indesirables</t>
+  </si>
+  <si>
+    <t>CorpsDocument.facteursDeRisqueProfessionnelsNonCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrFacteursDeRisqueProfessionnelsNonCode
 </t>
   </si>
   <si>
-    <t>Section Documents ajoutés</t>
-  </si>
-  <si>
-    <t>CorpsDocument.educationPatient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/EducationPatient
+    <t>Section Facteurs de risque professionnels non Codé</t>
+  </si>
+  <si>
+    <t>CorpsDocument.fonctionsPhysiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrFonctionsPhysiques
 </t>
   </si>
   <si>
-    <t>Section Education du patient</t>
-  </si>
-  <si>
-    <t>CorpsDocument.effetsIndesirables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/EffetsIndesirables
+    <t>Section Fonctions physiques</t>
+  </si>
+  <si>
+    <t>CorpsDocument.habitusModeDeVie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrHabitusModeDeVie
 </t>
   </si>
   <si>
-    <t>Section Effets indesirables</t>
-  </si>
-  <si>
-    <t>CorpsDocument.facteursDeRisqueProfessionnelsNonCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FacteursDeRisqueProfessionnelsNonCode
+    <t>Section Habitus et modes de vie</t>
+  </si>
+  <si>
+    <t>CorpsDocument.historiqueDesActes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrHistoriqueDesActes
 </t>
   </si>
   <si>
-    <t>Section Facteurs de risque professionnels non Codé</t>
-  </si>
-  <si>
-    <t>CorpsDocument.fonctionsPhysiques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FonctionsPhysiques
+    <t>Section Historique des actes</t>
+  </si>
+  <si>
+    <t>CorpsDocument.historiqueDesGrossesses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrHistoriqueDesGrossesses
 </t>
   </si>
   <si>
-    <t>Section Fonctions physiques</t>
-  </si>
-  <si>
-    <t>CorpsDocument.habitusModeDeVie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/HabitusModeDeVie
+    <t>Section Historique des grossesses</t>
+  </si>
+  <si>
+    <t>CorpsDocument.planSoins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrPlanSoins
 </t>
   </si>
   <si>
-    <t>Section Habitus et modes de vie</t>
-  </si>
-  <si>
-    <t>CorpsDocument.historiqueDesActes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/HistoriqueDesActes
+    <t>Section Plan de Soins</t>
+  </si>
+  <si>
+    <t>CorpsDocument.pointsDeVigilancesNonCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrPointsDeVigilancesNonCode
 </t>
   </si>
   <si>
-    <t>Section Historique des actes</t>
-  </si>
-  <si>
-    <t>CorpsDocument.historiqueDesGrossesses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/HistoriqueDesGrossesses
+    <t>Section Points de Vigilances non code</t>
+  </si>
+  <si>
+    <t>CorpsDocument.prescriptionDispositifsMedicaux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrPrescriptionDispositifsMedicaux
 </t>
   </si>
   <si>
-    <t>Section Historique des grossesses</t>
-  </si>
-  <si>
-    <t>CorpsDocument.planSoins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PlanSoins
+    <t>Section Prescription de dispositifs médicaux</t>
+  </si>
+  <si>
+    <t>CorpsDocument.prescriptionMedicaments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrPrescriptionMedicaments
 </t>
   </si>
   <si>
-    <t>Section Plan de Soins</t>
-  </si>
-  <si>
-    <t>CorpsDocument.pointsDeVigilancesNonCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PointsDeVigilancesNonCode
+    <t>Section Prescription médicaments</t>
+  </si>
+  <si>
+    <t>CorpsDocument.problemesActifs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrProblemesActifs
 </t>
   </si>
   <si>
-    <t>Section Points de Vigilances non code</t>
-  </si>
-  <si>
-    <t>CorpsDocument.prescriptionDispositifsMedicaux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PrescriptionDispositifsMedicaux
+    <t>Section Problemès Actifs</t>
+  </si>
+  <si>
+    <t>CorpsDocument.raisonRecommandationNonCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrRaisonRecommandationNonCode
 </t>
   </si>
   <si>
-    <t>Section Prescription de dispositifs médicaux</t>
-  </si>
-  <si>
-    <t>CorpsDocument.prescriptionMedicaments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PrescriptionMedicaments
+    <t>Section Raison de la recommandation (non Codé)</t>
+  </si>
+  <si>
+    <t>CorpsDocument.raisonRecommandation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrRaisonRecommandation
 </t>
   </si>
   <si>
-    <t>Section Prescription médicaments</t>
-  </si>
-  <si>
-    <t>CorpsDocument.problemesActifs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/ProblemesActifs
+    <t>Section Raison de la recommandation</t>
+  </si>
+  <si>
+    <t>CorpsDocument.resultatsLaboratoireBiologieSecondeIntention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrResultatsLaboratoireBiologieSecondeIntention
 </t>
   </si>
   <si>
-    <t>Section Problemès Actifs</t>
-  </si>
-  <si>
-    <t>CorpsDocument.raisonRecommandationNonCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/RaisonRecommandationNonCode
+    <t>Section Résultats de laboratoire de biologie de seconde intention</t>
+  </si>
+  <si>
+    <t>CorpsDocument.resultatsEvenements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrResultatsEvenements
 </t>
   </si>
   <si>
-    <t>Section Raison de la recommandation (non Codé)</t>
-  </si>
-  <si>
-    <t>CorpsDocument.raisonRecommandation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/RaisonRecommandation
+    <t>Section Resultats d'évenements</t>
+  </si>
+  <si>
+    <t>CorpsDocument.resultatsExamensNonCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrResultatsExamensNonCode
 </t>
   </si>
   <si>
-    <t>Section Raison de la recommandation</t>
-  </si>
-  <si>
-    <t>CorpsDocument.resultatsLaboratoireBiologieSecondeIntention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/ResultatsLaboratoireBiologieSecondeIntention
+    <t>Section Resultats d'xamens (non Codée)</t>
+  </si>
+  <si>
+    <t>CorpsDocument.resultatsExamens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrResultatsExamens
 </t>
   </si>
   <si>
-    <t>Section Résultats de laboratoire de biologie de seconde intention</t>
-  </si>
-  <si>
-    <t>CorpsDocument.resultatsEvenements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/ResultatsEvenements
+    <t>Section Résultats d'examens</t>
+  </si>
+  <si>
+    <t>CorpsDocument.resultats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrResultats
 </t>
   </si>
   <si>
-    <t>Section Resultats d'évenements</t>
-  </si>
-  <si>
-    <t>CorpsDocument.resultatsExamensNonCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/ResultatsExamensNonCode
+    <t>Section Resultats</t>
+  </si>
+  <si>
+    <t>CorpsDocument.signesVitaux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrSignesVitaux
 </t>
   </si>
   <si>
-    <t>Section Resultats d'xamens (non Codée)</t>
-  </si>
-  <si>
-    <t>CorpsDocument.resultatsExamens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/ResultatsExamens
+    <t>Section Signes vitaux</t>
+  </si>
+  <si>
+    <t>CorpsDocument.statutDocument</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrStatutDocument
 </t>
   </si>
   <si>
-    <t>Section Résultats d'examens</t>
-  </si>
-  <si>
-    <t>CorpsDocument.resultats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Resultats
+    <t>Section Statut du document</t>
+  </si>
+  <si>
+    <t>CorpsDocument.statutFonctionnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrStatutFonctionnel
 </t>
   </si>
   <si>
-    <t>Section Resultats</t>
-  </si>
-  <si>
-    <t>CorpsDocument.signesVitaux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/SignesVitaux
+    <t>Section Statut fonctionnel</t>
+  </si>
+  <si>
+    <t>CorpsDocument.traitements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrTraitement
 </t>
   </si>
   <si>
-    <t>Section Signes vitaux</t>
-  </si>
-  <si>
-    <t>CorpsDocument.statutDocument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/StatutDocument
+    <t>Section Traitement</t>
+  </si>
+  <si>
+    <t>CorpsDocument.traitementSortie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrTraitementSortie
 </t>
   </si>
   <si>
-    <t>Section Statut du document</t>
-  </si>
-  <si>
-    <t>CorpsDocument.statutFonctionnel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/StatutFonctionnel
+    <t>Section Traitement à la sortie</t>
+  </si>
+  <si>
+    <t>CorpsDocument.traitementsAdministres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrTraitementsAdministres
 </t>
   </si>
   <si>
-    <t>Section Statut fonctionnel</t>
-  </si>
-  <si>
-    <t>CorpsDocument.traitements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Traitement
-</t>
-  </si>
-  <si>
-    <t>Section Traitement</t>
-  </si>
-  <si>
-    <t>CorpsDocument.traitementSortie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/TraitementSortie
-</t>
-  </si>
-  <si>
-    <t>Section Traitement à la sortie</t>
-  </si>
-  <si>
-    <t>CorpsDocument.traitementsAdministres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/TraitementsAdministres
-</t>
-  </si>
-  <si>
     <t>Section Traitements administrés</t>
   </si>
   <si>
     <t>CorpsDocument.vaccinations</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Vaccinations
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/FrVaccinations
 </t>
   </si>
   <si>
@@ -1036,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ51"/>
+  <dimension ref="A1:AJ48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="50.05078125" customWidth="true" bestFit="true"/>
@@ -1049,7 +1019,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="90.91015625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="92.4609375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -5886,306 +5856,6 @@
         <v>72</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="N51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>72</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>